<commit_message>
a910: 双 ALU + 双 AIQ (AIQ1 与 MD 共用 pipe2 RR); 同步当前工作树
- IDU: AIQ 拆成 2×8 项, 平衡轮转派遣; AIQ1 发射 stall + rf_ctrl valid 保持;
  PRF 加 2 个读口; AIQ0 实例名保留 (difftest PERF 探针)
- IU: 新增 IU_wb_arb (严格 RR); IU_alu_pipe 加 wb_grant/wb_req/issue_stall;
  IU_md_pipe 输出加 2 项 skid (空时旁路), md_unit_stall 用下一拍占用
- A910: ALU1 (完成口 1) 写回与 MD 共用 pipe2; 五字段同源 mux;
  删除 difftest/smoke TB 对 cmplt_vld1/iid1 的 force (否则完成被吞、ROB 卡死)
- 回归: a910-difftest-all 46 PASS / 2 已知 FAIL; aiq-equiv 20 万拍 0 分歧;
  idu-unit / iu-alu-unit / iu-md-unit / iu-wb-arb-unit 全绿;
  coremark_i1 385,219 -> 369,187 拍 (-4.16%);
  整场 B IFU3: 3.894 / 256,752 cycles/iter (改前 3.744 / 267,049)
- 一并提交工作树中已完成的 IFU3 / LSIQ 参数化 / NPU / 文档等改动

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/rtu_接口对照表.xlsx
+++ b/doc/rtu_接口对照表.xlsx
@@ -2442,7 +2442,7 @@
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">SQ_ENTRY=6 / SDIQ_ENTRY=4 / LSIQ_ENTRY=8</t>
+          <t xml:space="preserve">SQ_ENTRY=6 / SDIQ_ENTRY=4 / LSIQ_ENTRY=12</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -2452,7 +2452,7 @@
       </c>
       <c r="G27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">2026-10-08 核过的实际档位（`lsu_top.sv:3-5`）：`SQ_ENTRY = 6` ⇒ 槽号 0..5 正好 3 位，**与 RTU 的 `disp*_sq_id[2:0]` 严丝合缝**；`SDIQ_ENTRY = 4`（对 IDU 的 `idu_lsu_st_sdiq_entry[3:0]`）；`LSIQ_ENTRY = 8`（对 IDU 的 `idu_lsu_ld/st_lch_entry[7:0]`）。⚠️ **旧文档正文里写的 `LSIQ_ENTRY = 12` 已过期** —— 2026-10-08 的 commit 165dfd5 "位宽对齐 64 preg / 8 LSIQ" 已把它改成 8。RTU 只用 `sq_id`，与 LSIQ 深度无关</t>
+          <t xml:space="preserve">`SQ_ENTRY = 6` ⇒ 槽号 0..5 正好 3 位，**与 RTU 的 `disp*_sq_id[2:0]` 严丝合缝**；`SDIQ_ENTRY = 4`（对 IDU 的 `idu_lsu_st_sdiq_entry[3:0]`）。⚠️ **`LSIQ_ENTRY` 的历史是 12 → 8 → 12**：2026-10-08 的 commit 165dfd5 "位宽对齐 64 preg / 8 LSIQ" 曾把它砍到 8；2026-10-16 按 C910 原版深度放回 **12**（`mySoC/lsiq_defines.vh` 是真源，IDU 的 `idu_lsu_ld/st_lch_entry` 现在是 `[11:0]`）。RTU 只用 `sq_id`，与 LSIQ 深度无关 —— 这条留着是提醒别再照抄旧数</t>
         </is>
       </c>
     </row>

</xml_diff>